<commit_message>
changed to GDD mode, bug in pyaquacrop package (mode flag should be opposite as described in the file)
</commit_message>
<xml_diff>
--- a/data/external/yield/maize/Podatki IOSDV - koruza za zrnje.xlsx
+++ b/data/external/yield/maize/Podatki IOSDV - koruza za zrnje.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rokku\Documents\Code\aquacrop-slovenia\data\external\yield\maize\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EDB7665-046B-48EE-9AF1-7CF0360C6B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF16B23A-9552-4442-92B9-7182A6E77496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44970" yWindow="690" windowWidth="27270" windowHeight="18765" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="47085" yWindow="1425" windowWidth="26370" windowHeight="18765" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="3" r:id="rId1"/>
@@ -8752,23 +8752,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="dd965b64-2411-47f7-89d5-218539f846c5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004E18FDA38211884689C972839BBE4E93" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d79fa8820f456ca99f0dc5e5e4bab8cc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="dd965b64-2411-47f7-89d5-218539f846c5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d24846eac545d96bd52d4a7e416c480b" ns3:_="">
     <xsd:import namespace="dd965b64-2411-47f7-89d5-218539f846c5"/>
@@ -8962,31 +8945,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71DE8921-2C6F-47FD-B08D-3AA8A450D9E8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="dd965b64-2411-47f7-89d5-218539f846c5"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{902540C8-10AC-475C-8811-3255CA7A7D4A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="dd965b64-2411-47f7-89d5-218539f846c5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C8E1E15-75CC-42AE-86C3-0B6EBA8ED4CA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9002,4 +8978,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{902540C8-10AC-475C-8811-3255CA7A7D4A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71DE8921-2C6F-47FD-B08D-3AA8A450D9E8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="dd965b64-2411-47f7-89d5-218539f846c5"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>